<commit_message>
Update manual fund chart inputs
</commit_message>
<xml_diff>
--- a/Hana_EMP.xlsx
+++ b/Hana_EMP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\infomax\Documents\Codex\펀드차트\fund_returns_daily\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A514A749-1A99-4FD9-B861-44F11305D408}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB24C665-8D59-47B5-AA30-26F64D6F3792}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="390" yWindow="390" windowWidth="15960" windowHeight="14985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -111,12 +111,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -142,7 +148,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -173,6 +179,36 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -558,7 +594,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:S385"/>
+  <dimension ref="A1:S403"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.125" customWidth="1"/>
@@ -8825,11 +8861,11 @@
         <v>0.1973</v>
       </c>
       <c r="D370" s="7">
-        <f t="shared" ref="D370" si="395">D$246+I370</f>
+        <f>D$246+I370</f>
         <v>0.15129999999999999</v>
       </c>
       <c r="E370" s="4">
-        <f t="shared" ref="E370" si="396">E$246+J370</f>
+        <f t="shared" ref="E370" si="395">E$246+J370</f>
         <v>6.4399999999999999E-2</v>
       </c>
       <c r="G370" s="9">
@@ -8853,19 +8889,19 @@
         <v>46211</v>
       </c>
       <c r="B371" s="4">
-        <f t="shared" ref="B371" si="397">B$246+G371</f>
+        <f t="shared" ref="B371" si="396">B$246+G371</f>
         <v>0.24819999999999998</v>
       </c>
       <c r="C371" s="7">
-        <f t="shared" ref="C371:C381" si="398">C$246+H371+$L$370</f>
+        <f>C$246+H371+$L$370</f>
         <v>0.19729999999999998</v>
       </c>
       <c r="D371" s="7">
-        <f t="shared" ref="D371" si="399">D$246+I371</f>
+        <f t="shared" ref="D371" si="397">D$246+I371</f>
         <v>0.14360000000000001</v>
       </c>
       <c r="E371" s="4">
-        <f t="shared" ref="E371" si="400">E$246+J371</f>
+        <f t="shared" ref="E371" si="398">E$246+J371</f>
         <v>5.3400000000000003E-2</v>
       </c>
       <c r="G371" s="9">
@@ -8887,19 +8923,19 @@
         <v>46212</v>
       </c>
       <c r="B372" s="4">
-        <f t="shared" ref="B372" si="401">B$246+G372</f>
+        <f t="shared" ref="B372" si="399">B$246+G372</f>
         <v>0.24529999999999999</v>
       </c>
       <c r="C372" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" ref="C371:C381" si="400">C$246+H372+$L$370</f>
         <v>0.18790000000000001</v>
       </c>
       <c r="D372" s="7">
-        <f t="shared" ref="D372" si="402">D$246+I372</f>
+        <f t="shared" ref="D372" si="401">D$246+I372</f>
         <v>0.14300000000000002</v>
       </c>
       <c r="E372" s="4">
-        <f t="shared" ref="E372" si="403">E$246+J372</f>
+        <f t="shared" ref="E372" si="402">E$246+J372</f>
         <v>5.33E-2</v>
       </c>
       <c r="G372" s="9">
@@ -8921,19 +8957,19 @@
         <v>46213</v>
       </c>
       <c r="B373" s="4">
-        <f t="shared" ref="B373" si="404">B$246+G373</f>
+        <f t="shared" ref="B373" si="403">B$246+G373</f>
         <v>0.24909999999999999</v>
       </c>
       <c r="C373" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.19450000000000001</v>
       </c>
       <c r="D373" s="7">
-        <f t="shared" ref="D373" si="405">D$246+I373</f>
+        <f t="shared" ref="D373" si="404">D$246+I373</f>
         <v>0.14929999999999999</v>
       </c>
       <c r="E373" s="4">
-        <f t="shared" ref="E373" si="406">E$246+J373</f>
+        <f t="shared" ref="E373" si="405">E$246+J373</f>
         <v>5.6399999999999999E-2</v>
       </c>
       <c r="G373" s="9">
@@ -8958,19 +8994,19 @@
         <v>46216</v>
       </c>
       <c r="B374" s="4">
-        <f t="shared" ref="B374" si="407">B$246+G374</f>
+        <f t="shared" ref="B374" si="406">B$246+G374</f>
         <v>0.25180000000000002</v>
       </c>
       <c r="C374" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.1956</v>
       </c>
       <c r="D374" s="7">
-        <f t="shared" ref="D374" si="408">D$246+I374</f>
+        <f t="shared" ref="D374" si="407">D$246+I374</f>
         <v>0.15060000000000001</v>
       </c>
       <c r="E374" s="4">
-        <f t="shared" ref="E374:E381" si="409">E$246+J374+$N$374</f>
+        <f>E$246+J374+$N$374</f>
         <v>4.7300000000000002E-2</v>
       </c>
       <c r="G374" s="9">
@@ -8995,19 +9031,19 @@
         <v>46217</v>
       </c>
       <c r="B375" s="4">
-        <f t="shared" ref="B375" si="410">B$246+G375</f>
+        <f t="shared" ref="B375" si="408">B$246+G375</f>
         <v>0.24679999999999999</v>
       </c>
       <c r="C375" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.18240000000000001</v>
       </c>
       <c r="D375" s="7">
-        <f t="shared" ref="D375" si="411">D$246+I375</f>
+        <f t="shared" ref="D375" si="409">D$246+I375</f>
         <v>0.14150000000000001</v>
       </c>
       <c r="E375" s="4">
-        <f t="shared" si="409"/>
+        <f t="shared" ref="E374:E381" si="410">E$246+J375+$N$374</f>
         <v>4.5700000000000005E-2</v>
       </c>
       <c r="G375" s="9">
@@ -9030,19 +9066,19 @@
         <v>46218</v>
       </c>
       <c r="B376" s="4">
-        <f t="shared" ref="B376" si="412">B$246+G376</f>
+        <f t="shared" ref="B376" si="411">B$246+G376</f>
         <v>0.251</v>
       </c>
       <c r="C376" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.19019999999999998</v>
       </c>
       <c r="D376" s="7">
-        <f t="shared" ref="D376" si="413">D$246+I376</f>
+        <f t="shared" ref="D376" si="412">D$246+I376</f>
         <v>0.1464</v>
       </c>
       <c r="E376" s="4">
-        <f t="shared" si="409"/>
+        <f t="shared" si="410"/>
         <v>4.8500000000000001E-2</v>
       </c>
       <c r="G376" s="9">
@@ -9065,19 +9101,19 @@
         <v>46219</v>
       </c>
       <c r="B377" s="4">
-        <f t="shared" ref="B377" si="414">B$246+G377</f>
+        <f t="shared" ref="B377" si="413">B$246+G377</f>
         <v>0.25329999999999997</v>
       </c>
       <c r="C377" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.1895</v>
       </c>
       <c r="D377" s="7">
-        <f t="shared" ref="D377" si="415">D$246+I377</f>
+        <f t="shared" ref="D377" si="414">D$246+I377</f>
         <v>0.1484</v>
       </c>
       <c r="E377" s="4">
-        <f t="shared" si="409"/>
+        <f t="shared" si="410"/>
         <v>4.5700000000000005E-2</v>
       </c>
       <c r="G377" s="9">
@@ -9100,19 +9136,19 @@
         <v>46223</v>
       </c>
       <c r="B378" s="4">
-        <f t="shared" ref="B378" si="416">B$246+G378</f>
+        <f t="shared" ref="B378" si="415">B$246+G378</f>
         <v>0.24390000000000001</v>
       </c>
       <c r="C378" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.17609999999999998</v>
       </c>
       <c r="D378" s="7">
-        <f t="shared" ref="D378" si="417">D$246+I378</f>
+        <f t="shared" ref="D378" si="416">D$246+I378</f>
         <v>0.13830000000000001</v>
       </c>
       <c r="E378" s="4">
-        <f t="shared" si="409"/>
+        <f t="shared" si="410"/>
         <v>3.5799999999999998E-2</v>
       </c>
       <c r="G378" s="9">
@@ -9135,19 +9171,19 @@
         <v>46224</v>
       </c>
       <c r="B379" s="4">
-        <f t="shared" ref="B379" si="418">B$246+G379</f>
+        <f t="shared" ref="B379" si="417">B$246+G379</f>
         <v>0.24299999999999999</v>
       </c>
       <c r="C379" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.1749</v>
       </c>
       <c r="D379" s="7">
-        <f t="shared" ref="D379" si="419">D$246+I379</f>
+        <f t="shared" ref="D379" si="418">D$246+I379</f>
         <v>0.13519999999999999</v>
       </c>
       <c r="E379" s="4">
-        <f t="shared" si="409"/>
+        <f t="shared" si="410"/>
         <v>3.9800000000000002E-2</v>
       </c>
       <c r="G379" s="9">
@@ -9170,19 +9206,19 @@
         <v>46225</v>
       </c>
       <c r="B380" s="4">
-        <f t="shared" ref="B380" si="420">B$246+G380</f>
+        <f t="shared" ref="B380" si="419">B$246+G380</f>
         <v>0.24959999999999999</v>
       </c>
       <c r="C380" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.18530000000000002</v>
       </c>
       <c r="D380" s="7">
-        <f t="shared" ref="D380" si="421">D$246+I380</f>
+        <f t="shared" ref="D380" si="420">D$246+I380</f>
         <v>0.14250000000000002</v>
       </c>
       <c r="E380" s="4">
-        <f t="shared" si="409"/>
+        <f t="shared" si="410"/>
         <v>4.53E-2</v>
       </c>
       <c r="G380" s="9">
@@ -9205,19 +9241,19 @@
         <v>46226</v>
       </c>
       <c r="B381" s="4">
-        <f t="shared" ref="B381" si="422">B$246+G381</f>
+        <f t="shared" ref="B381" si="421">B$246+G381</f>
         <v>0.24919999999999998</v>
       </c>
       <c r="C381" s="7">
-        <f t="shared" si="398"/>
+        <f t="shared" si="400"/>
         <v>0.184</v>
       </c>
       <c r="D381" s="7">
-        <f t="shared" ref="D381" si="423">D$246+I381</f>
+        <f t="shared" ref="D381" si="422">D$246+I381</f>
         <v>0.14019999999999999</v>
       </c>
       <c r="E381" s="4">
-        <f t="shared" si="409"/>
+        <f t="shared" si="410"/>
         <v>4.4999999999999998E-2</v>
       </c>
       <c r="G381" s="9">
@@ -9240,19 +9276,19 @@
         <v>46227</v>
       </c>
       <c r="B382" s="4">
-        <f t="shared" ref="B382" si="424">B$246+G382</f>
+        <f t="shared" ref="B382" si="423">B$246+G382</f>
         <v>0.245</v>
       </c>
       <c r="C382" s="7">
-        <f t="shared" ref="C382" si="425">C$246+H382+$L$370</f>
+        <f t="shared" ref="C382" si="424">C$246+H382+$L$370</f>
         <v>0.18109999999999998</v>
       </c>
       <c r="D382" s="7">
-        <f t="shared" ref="D382" si="426">D$246+I382</f>
+        <f t="shared" ref="D382" si="425">D$246+I382</f>
         <v>0.1338</v>
       </c>
       <c r="E382" s="4">
-        <f t="shared" ref="E382" si="427">E$246+J382+$N$374</f>
+        <f t="shared" ref="E382" si="426">E$246+J382+$N$374</f>
         <v>3.6500000000000005E-2</v>
       </c>
       <c r="G382" s="9">
@@ -9275,19 +9311,19 @@
         <v>46230</v>
       </c>
       <c r="B383" s="4">
-        <f t="shared" ref="B383" si="428">B$246+G383</f>
+        <f t="shared" ref="B383" si="427">B$246+G383</f>
         <v>0.24440000000000001</v>
       </c>
       <c r="C383" s="7">
-        <f t="shared" ref="C383" si="429">C$246+H383+$L$370</f>
+        <f t="shared" ref="C383" si="428">C$246+H383+$L$370</f>
         <v>0.17649999999999999</v>
       </c>
       <c r="D383" s="7">
-        <f t="shared" ref="D383" si="430">D$246+I383</f>
+        <f t="shared" ref="D383" si="429">D$246+I383</f>
         <v>0.1338</v>
       </c>
       <c r="E383" s="4">
-        <f t="shared" ref="E383" si="431">E$246+J383+$N$374</f>
+        <f t="shared" ref="E383" si="430">E$246+J383+$N$374</f>
         <v>4.0800000000000003E-2</v>
       </c>
       <c r="G383" s="9">
@@ -9310,19 +9346,19 @@
         <v>46231</v>
       </c>
       <c r="B384" s="4">
-        <f t="shared" ref="B384" si="432">B$246+G384</f>
+        <f t="shared" ref="B384" si="431">B$246+G384</f>
         <v>0.24299999999999999</v>
       </c>
       <c r="C384" s="7">
-        <f t="shared" ref="C384" si="433">C$246+H384+$L$370</f>
+        <f t="shared" ref="C384" si="432">C$246+H384+$L$370</f>
         <v>0.17620000000000002</v>
       </c>
       <c r="D384" s="7">
-        <f t="shared" ref="D384" si="434">D$246+I384</f>
+        <f t="shared" ref="D384" si="433">D$246+I384</f>
         <v>0.1361</v>
       </c>
       <c r="E384" s="4">
-        <f t="shared" ref="E384" si="435">E$246+J384+$N$374</f>
+        <f t="shared" ref="E384" si="434">E$246+J384+$N$374</f>
         <v>3.1899999999999998E-2</v>
       </c>
       <c r="G384" s="9">
@@ -9345,19 +9381,19 @@
         <v>46232</v>
       </c>
       <c r="B385" s="4">
-        <f t="shared" ref="B385" si="436">B$246+G385</f>
+        <f t="shared" ref="B385" si="435">B$246+G385</f>
         <v>0.2419</v>
       </c>
       <c r="C385" s="7">
-        <f t="shared" ref="C385" si="437">C$246+H385+$L$370</f>
+        <f t="shared" ref="C385" si="436">C$246+H385+$L$370</f>
         <v>0.17049999999999998</v>
       </c>
       <c r="D385" s="7">
-        <f t="shared" ref="D385" si="438">D$246+I385</f>
+        <f t="shared" ref="D385" si="437">D$246+I385</f>
         <v>0.1363</v>
       </c>
       <c r="E385" s="4">
-        <f t="shared" ref="E385" si="439">E$246+J385+$N$374</f>
+        <f t="shared" ref="E385" si="438">E$246+J385+$N$374</f>
         <v>2.7099999999999999E-2</v>
       </c>
       <c r="G385" s="9">
@@ -9374,6 +9410,640 @@
       </c>
       <c r="L385" s="9"/>
       <c r="N385" s="9"/>
+    </row>
+    <row r="386" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A386" s="3">
+        <v>46233</v>
+      </c>
+      <c r="B386" s="4">
+        <f t="shared" ref="B386" si="439">B$246+G386</f>
+        <v>0.23669999999999999</v>
+      </c>
+      <c r="C386" s="7">
+        <f t="shared" ref="C386" si="440">C$246+H386+$L$370</f>
+        <v>0.1618</v>
+      </c>
+      <c r="D386" s="7">
+        <f t="shared" ref="D386" si="441">D$246+I386</f>
+        <v>0.12479999999999999</v>
+      </c>
+      <c r="E386" s="4">
+        <f t="shared" ref="E386" si="442">E$246+J386+$N$374</f>
+        <v>1.9300000000000001E-2</v>
+      </c>
+      <c r="G386" s="9">
+        <v>6.6799999999999998E-2</v>
+      </c>
+      <c r="H386" s="9">
+        <v>2.5100000000000001E-2</v>
+      </c>
+      <c r="I386" s="9">
+        <v>5.1000000000000004E-3</v>
+      </c>
+      <c r="J386" s="9">
+        <v>3.8E-3</v>
+      </c>
+      <c r="L386" s="9"/>
+      <c r="N386" s="9"/>
+    </row>
+    <row r="387" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A387" s="3">
+        <v>46234</v>
+      </c>
+      <c r="B387" s="4">
+        <f t="shared" ref="B387" si="443">B$246+G387</f>
+        <v>0.24479999999999999</v>
+      </c>
+      <c r="C387" s="7">
+        <f t="shared" ref="C387" si="444">C$246+H387+$L$370</f>
+        <v>0.1799</v>
+      </c>
+      <c r="D387" s="7">
+        <f t="shared" ref="D387" si="445">D$246+I387</f>
+        <v>0.13830000000000001</v>
+      </c>
+      <c r="E387" s="4">
+        <f t="shared" ref="E387" si="446">E$246+J387+$N$374</f>
+        <v>3.2399999999999998E-2</v>
+      </c>
+      <c r="G387" s="9">
+        <v>7.4899999999999994E-2</v>
+      </c>
+      <c r="H387" s="9">
+        <v>4.3200000000000002E-2</v>
+      </c>
+      <c r="I387" s="9">
+        <v>1.8599999999999998E-2</v>
+      </c>
+      <c r="J387" s="9">
+        <v>1.6899999999999998E-2</v>
+      </c>
+      <c r="L387" s="9"/>
+      <c r="N387" s="9"/>
+    </row>
+    <row r="388" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A388" s="3">
+        <v>46237</v>
+      </c>
+      <c r="B388" s="4">
+        <f t="shared" ref="B388" si="447">B$246+G388</f>
+        <v>0.24819999999999998</v>
+      </c>
+      <c r="C388" s="7">
+        <f t="shared" ref="C388" si="448">C$246+H388+$L$370</f>
+        <v>0.18099999999999999</v>
+      </c>
+      <c r="D388" s="7">
+        <f t="shared" ref="D388" si="449">D$246+I388</f>
+        <v>0.1394</v>
+      </c>
+      <c r="E388" s="4">
+        <f t="shared" ref="E388" si="450">E$246+J388+$N$374</f>
+        <v>3.27E-2</v>
+      </c>
+      <c r="G388" s="9">
+        <v>7.8299999999999995E-2</v>
+      </c>
+      <c r="H388" s="9">
+        <v>4.4299999999999999E-2</v>
+      </c>
+      <c r="I388" s="9">
+        <v>1.9699999999999999E-2</v>
+      </c>
+      <c r="J388" s="9">
+        <v>1.72E-2</v>
+      </c>
+      <c r="L388" s="9"/>
+      <c r="N388" s="9"/>
+    </row>
+    <row r="389" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A389" s="3">
+        <v>46238</v>
+      </c>
+      <c r="B389" s="4">
+        <f t="shared" ref="B389" si="451">B$246+G389</f>
+        <v>0.25319999999999998</v>
+      </c>
+      <c r="C389" s="7">
+        <f t="shared" ref="C389" si="452">C$246+H389+$L$370</f>
+        <v>0.18719999999999998</v>
+      </c>
+      <c r="D389" s="7">
+        <f t="shared" ref="D389" si="453">D$246+I389</f>
+        <v>0.1469</v>
+      </c>
+      <c r="E389" s="4">
+        <f t="shared" ref="E389" si="454">E$246+J389+$N$374</f>
+        <v>3.8199999999999998E-2</v>
+      </c>
+      <c r="G389" s="9">
+        <v>8.3299999999999999E-2</v>
+      </c>
+      <c r="H389" s="9">
+        <v>5.0500000000000003E-2</v>
+      </c>
+      <c r="I389" s="9">
+        <v>2.7199999999999998E-2</v>
+      </c>
+      <c r="J389" s="9">
+        <v>2.2700000000000001E-2</v>
+      </c>
+      <c r="L389" s="9"/>
+      <c r="N389" s="9"/>
+    </row>
+    <row r="390" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A390" s="3">
+        <v>46239</v>
+      </c>
+      <c r="B390" s="4">
+        <f t="shared" ref="B390" si="455">B$246+G390</f>
+        <v>0.26339999999999997</v>
+      </c>
+      <c r="C390" s="7">
+        <f t="shared" ref="C390" si="456">C$246+H390+$L$370</f>
+        <v>0.2031</v>
+      </c>
+      <c r="D390" s="7">
+        <f t="shared" ref="D390" si="457">D$246+I390</f>
+        <v>0.16159999999999999</v>
+      </c>
+      <c r="E390" s="4">
+        <f t="shared" ref="E390" si="458">E$246+J390+$N$374</f>
+        <v>4.9099999999999998E-2</v>
+      </c>
+      <c r="G390" s="9">
+        <v>9.35E-2</v>
+      </c>
+      <c r="H390" s="9">
+        <v>6.6400000000000001E-2</v>
+      </c>
+      <c r="I390" s="9">
+        <v>4.19E-2</v>
+      </c>
+      <c r="J390" s="9">
+        <v>3.3599999999999998E-2</v>
+      </c>
+      <c r="L390" s="9"/>
+      <c r="N390" s="9"/>
+    </row>
+    <row r="391" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A391" s="16">
+        <v>46240</v>
+      </c>
+      <c r="B391" s="17">
+        <f t="shared" ref="B391" si="459">B$246+G391</f>
+        <v>0.26290000000000002</v>
+      </c>
+      <c r="C391" s="18">
+        <f t="shared" ref="C391" si="460">C$246+H391+$L$370</f>
+        <v>0.20429999999999998</v>
+      </c>
+      <c r="D391" s="18">
+        <f t="shared" ref="D391" si="461">D$246+I391</f>
+        <v>0.16209999999999999</v>
+      </c>
+      <c r="E391" s="17">
+        <f t="shared" ref="E391" si="462">E$246+J391+$N$374</f>
+        <v>4.8800000000000003E-2</v>
+      </c>
+      <c r="F391" s="19"/>
+      <c r="G391" s="20">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="H391" s="20">
+        <v>6.7599999999999993E-2</v>
+      </c>
+      <c r="I391" s="20">
+        <v>4.24E-2</v>
+      </c>
+      <c r="J391" s="20">
+        <v>3.3300000000000003E-2</v>
+      </c>
+      <c r="L391" s="9"/>
+      <c r="N391" s="9"/>
+    </row>
+    <row r="392" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A392" s="11">
+        <v>46241</v>
+      </c>
+      <c r="B392" s="12">
+        <f t="shared" ref="B392" si="463">B$246+G392</f>
+        <v>0.2616</v>
+      </c>
+      <c r="C392" s="13">
+        <f t="shared" ref="C392" si="464">C$246+H392+$L$370</f>
+        <v>0.20169999999999999</v>
+      </c>
+      <c r="D392" s="13">
+        <f t="shared" ref="D392" si="465">D$246+I392</f>
+        <v>0.1585</v>
+      </c>
+      <c r="E392" s="12">
+        <f>E$246+J392+$N$374+$N$392</f>
+        <v>4.8399999999999999E-2</v>
+      </c>
+      <c r="F392" s="14"/>
+      <c r="G392" s="15">
+        <v>9.1700000000000004E-2</v>
+      </c>
+      <c r="H392" s="15">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="I392" s="15">
+        <v>3.8800000000000001E-2</v>
+      </c>
+      <c r="J392" s="15">
+        <v>2.6700000000000002E-2</v>
+      </c>
+      <c r="L392" s="9"/>
+      <c r="N392" s="9">
+        <v>6.1999999999999998E-3</v>
+      </c>
+    </row>
+    <row r="393" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A393" s="3">
+        <v>46244</v>
+      </c>
+      <c r="B393" s="4">
+        <f t="shared" ref="B393" si="466">B$246+G393</f>
+        <v>0.26679999999999998</v>
+      </c>
+      <c r="C393" s="7">
+        <f t="shared" ref="C393" si="467">C$246+H393+$L$370</f>
+        <v>0.20900000000000002</v>
+      </c>
+      <c r="D393" s="7">
+        <f t="shared" ref="D393" si="468">D$246+I393</f>
+        <v>0.1646</v>
+      </c>
+      <c r="E393" s="4">
+        <f>E$246+J393+$N$374+N392</f>
+        <v>5.2699999999999997E-2</v>
+      </c>
+      <c r="G393" s="9">
+        <v>9.69E-2</v>
+      </c>
+      <c r="H393" s="9">
+        <v>7.2300000000000003E-2</v>
+      </c>
+      <c r="I393" s="9">
+        <v>4.4900000000000002E-2</v>
+      </c>
+      <c r="J393" s="9">
+        <v>3.1E-2</v>
+      </c>
+      <c r="L393" s="9"/>
+      <c r="N393" s="9"/>
+    </row>
+    <row r="394" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A394" s="3">
+        <v>46245</v>
+      </c>
+      <c r="B394" s="4">
+        <f t="shared" ref="B394" si="469">B$246+G394</f>
+        <v>0.26700000000000002</v>
+      </c>
+      <c r="C394" s="7">
+        <f t="shared" ref="C394" si="470">C$246+H394+$L$370</f>
+        <v>0.20729999999999998</v>
+      </c>
+      <c r="D394" s="7">
+        <f t="shared" ref="D394" si="471">D$246+I394</f>
+        <v>0.16089999999999999</v>
+      </c>
+      <c r="E394" s="4">
+        <f>E$246+J394+$N$374+$N$392</f>
+        <v>5.4199999999999998E-2</v>
+      </c>
+      <c r="G394" s="9">
+        <v>9.7100000000000006E-2</v>
+      </c>
+      <c r="H394" s="9">
+        <v>7.0599999999999996E-2</v>
+      </c>
+      <c r="I394" s="9">
+        <v>4.1200000000000001E-2</v>
+      </c>
+      <c r="J394" s="9">
+        <v>3.2500000000000001E-2</v>
+      </c>
+      <c r="L394" s="9"/>
+      <c r="N394" s="9"/>
+    </row>
+    <row r="395" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A395" s="3">
+        <v>46246</v>
+      </c>
+      <c r="B395" s="4">
+        <f t="shared" ref="B395" si="472">B$246+G395</f>
+        <v>0.2666</v>
+      </c>
+      <c r="C395" s="7">
+        <f t="shared" ref="C395" si="473">C$246+H395+$L$370</f>
+        <v>0.20800000000000002</v>
+      </c>
+      <c r="D395" s="7">
+        <f t="shared" ref="D395" si="474">D$246+I395</f>
+        <v>0.16059999999999999</v>
+      </c>
+      <c r="E395" s="4">
+        <f t="shared" ref="E395:E402" si="475">E$246+J395+$N$374+$N$392</f>
+        <v>5.62E-2</v>
+      </c>
+      <c r="G395" s="9">
+        <v>9.6699999999999994E-2</v>
+      </c>
+      <c r="H395" s="9">
+        <v>7.1300000000000002E-2</v>
+      </c>
+      <c r="I395" s="9">
+        <v>4.0899999999999999E-2</v>
+      </c>
+      <c r="J395" s="9">
+        <v>3.4500000000000003E-2</v>
+      </c>
+      <c r="L395" s="9"/>
+      <c r="N395" s="9"/>
+    </row>
+    <row r="396" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A396" s="3">
+        <v>46247</v>
+      </c>
+      <c r="B396" s="4">
+        <f t="shared" ref="B396" si="476">B$246+G396</f>
+        <v>0.27010000000000001</v>
+      </c>
+      <c r="C396" s="7">
+        <f t="shared" ref="C396" si="477">C$246+H396+$L$370</f>
+        <v>0.21389999999999998</v>
+      </c>
+      <c r="D396" s="7">
+        <f t="shared" ref="D396" si="478">D$246+I396</f>
+        <v>0.1643</v>
+      </c>
+      <c r="E396" s="4">
+        <f t="shared" si="475"/>
+        <v>5.9399999999999994E-2</v>
+      </c>
+      <c r="G396" s="9">
+        <v>0.1002</v>
+      </c>
+      <c r="H396" s="9">
+        <v>7.7200000000000005E-2</v>
+      </c>
+      <c r="I396" s="9">
+        <v>4.4600000000000001E-2</v>
+      </c>
+      <c r="J396" s="9">
+        <v>3.7699999999999997E-2</v>
+      </c>
+      <c r="L396" s="9"/>
+      <c r="N396" s="9"/>
+    </row>
+    <row r="397" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A397" s="3">
+        <v>46248</v>
+      </c>
+      <c r="B397" s="4">
+        <f t="shared" ref="B397" si="479">B$246+G397</f>
+        <v>0.2747</v>
+      </c>
+      <c r="C397" s="7">
+        <f t="shared" ref="C397" si="480">C$246+H397+$L$370</f>
+        <v>0.21649999999999997</v>
+      </c>
+      <c r="D397" s="7">
+        <f t="shared" ref="D397" si="481">D$246+I397</f>
+        <v>0.16949999999999998</v>
+      </c>
+      <c r="E397" s="4">
+        <f t="shared" si="475"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="G397" s="9">
+        <v>0.1048</v>
+      </c>
+      <c r="H397" s="9">
+        <v>7.9799999999999996E-2</v>
+      </c>
+      <c r="I397" s="9">
+        <v>4.9799999999999997E-2</v>
+      </c>
+      <c r="J397" s="9">
+        <v>4.0800000000000003E-2</v>
+      </c>
+      <c r="L397" s="9"/>
+      <c r="N397" s="9"/>
+    </row>
+    <row r="398" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A398" s="3">
+        <v>46252</v>
+      </c>
+      <c r="B398" s="4">
+        <f t="shared" ref="B398" si="482">B$246+G398</f>
+        <v>0.27289999999999998</v>
+      </c>
+      <c r="C398" s="7">
+        <f t="shared" ref="C398" si="483">C$246+H398+$L$370</f>
+        <v>0.21739999999999998</v>
+      </c>
+      <c r="D398" s="7">
+        <f t="shared" ref="D398" si="484">D$246+I398</f>
+        <v>0.1651</v>
+      </c>
+      <c r="E398" s="4">
+        <f t="shared" si="475"/>
+        <v>6.2E-2</v>
+      </c>
+      <c r="G398" s="9">
+        <v>0.10299999999999999</v>
+      </c>
+      <c r="H398" s="9">
+        <v>8.0699999999999994E-2</v>
+      </c>
+      <c r="I398" s="9">
+        <v>4.5400000000000003E-2</v>
+      </c>
+      <c r="J398" s="9">
+        <v>4.0300000000000002E-2</v>
+      </c>
+      <c r="L398" s="9"/>
+      <c r="N398" s="9"/>
+    </row>
+    <row r="399" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A399" s="3">
+        <v>46253</v>
+      </c>
+      <c r="B399" s="4">
+        <f t="shared" ref="B399" si="485">B$246+G399</f>
+        <v>0.26729999999999998</v>
+      </c>
+      <c r="C399" s="7">
+        <f t="shared" ref="C399" si="486">C$246+H399+$L$370</f>
+        <v>0.2056</v>
+      </c>
+      <c r="D399" s="7">
+        <f t="shared" ref="D399" si="487">D$246+I399</f>
+        <v>0.15789999999999998</v>
+      </c>
+      <c r="E399" s="4">
+        <f t="shared" si="475"/>
+        <v>5.0499999999999996E-2</v>
+      </c>
+      <c r="G399" s="9">
+        <v>9.74E-2</v>
+      </c>
+      <c r="H399" s="9">
+        <v>6.8900000000000003E-2</v>
+      </c>
+      <c r="I399" s="9">
+        <v>3.8199999999999998E-2</v>
+      </c>
+      <c r="J399" s="9">
+        <v>2.8799999999999999E-2</v>
+      </c>
+      <c r="L399" s="9"/>
+      <c r="N399" s="9"/>
+    </row>
+    <row r="400" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A400" s="3">
+        <v>46254</v>
+      </c>
+      <c r="B400" s="4">
+        <f t="shared" ref="B400" si="488">B$246+G400</f>
+        <v>0.27239999999999998</v>
+      </c>
+      <c r="C400" s="7">
+        <f t="shared" ref="C400" si="489">C$246+H400+$L$370</f>
+        <v>0.21060000000000001</v>
+      </c>
+      <c r="D400" s="7">
+        <f t="shared" ref="D400" si="490">D$246+I400</f>
+        <v>0.16289999999999999</v>
+      </c>
+      <c r="E400" s="4">
+        <f t="shared" si="475"/>
+        <v>5.7099999999999998E-2</v>
+      </c>
+      <c r="G400" s="9">
+        <v>0.10249999999999999</v>
+      </c>
+      <c r="H400" s="9">
+        <v>7.3899999999999993E-2</v>
+      </c>
+      <c r="I400" s="9">
+        <v>4.3200000000000002E-2</v>
+      </c>
+      <c r="J400" s="9">
+        <v>3.5400000000000001E-2</v>
+      </c>
+      <c r="L400" s="9"/>
+      <c r="N400" s="9"/>
+    </row>
+    <row r="401" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A401" s="3">
+        <v>46255</v>
+      </c>
+      <c r="B401" s="4">
+        <f t="shared" ref="B401" si="491">B$246+G401</f>
+        <v>0.26960000000000001</v>
+      </c>
+      <c r="C401" s="7">
+        <f t="shared" ref="C401" si="492">C$246+H401+$L$370</f>
+        <v>0.20800000000000002</v>
+      </c>
+      <c r="D401" s="7">
+        <f t="shared" ref="D401" si="493">D$246+I401</f>
+        <v>0.1578</v>
+      </c>
+      <c r="E401" s="4">
+        <f t="shared" si="475"/>
+        <v>5.4099999999999995E-2</v>
+      </c>
+      <c r="G401" s="9">
+        <v>9.9699999999999997E-2</v>
+      </c>
+      <c r="H401" s="9">
+        <v>7.1300000000000002E-2</v>
+      </c>
+      <c r="I401" s="9">
+        <v>3.8100000000000002E-2</v>
+      </c>
+      <c r="J401" s="9">
+        <v>3.2399999999999998E-2</v>
+      </c>
+      <c r="L401" s="9"/>
+      <c r="N401" s="9"/>
+    </row>
+    <row r="402" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A402" s="3">
+        <v>46258</v>
+      </c>
+      <c r="B402" s="4">
+        <f t="shared" ref="B402" si="494">B$246+G402</f>
+        <v>0.27229999999999999</v>
+      </c>
+      <c r="C402" s="7">
+        <f>C$246+H402+$L$370</f>
+        <v>0.21150000000000002</v>
+      </c>
+      <c r="D402" s="7">
+        <f t="shared" ref="D402" si="495">D$246+I402</f>
+        <v>0.16120000000000001</v>
+      </c>
+      <c r="E402" s="4">
+        <f>E$246+J402+$N$374+$N$392</f>
+        <v>5.4699999999999999E-2</v>
+      </c>
+      <c r="G402" s="9">
+        <v>0.1024</v>
+      </c>
+      <c r="H402" s="9">
+        <v>7.4800000000000005E-2</v>
+      </c>
+      <c r="I402" s="9">
+        <v>4.1500000000000002E-2</v>
+      </c>
+      <c r="J402" s="9">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="L402" s="9"/>
+      <c r="N402" s="9"/>
+    </row>
+    <row r="403" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A403" s="3">
+        <v>46259</v>
+      </c>
+      <c r="B403" s="4">
+        <f t="shared" ref="B403" si="496">B$246+G403</f>
+        <v>0.27090000000000003</v>
+      </c>
+      <c r="C403" s="7">
+        <f>C$246+H403+$L$370</f>
+        <v>0.20739999999999997</v>
+      </c>
+      <c r="D403" s="7">
+        <f t="shared" ref="D403" si="497">D$246+I403</f>
+        <v>0.1595</v>
+      </c>
+      <c r="E403" s="4">
+        <f>E$246+J403+$N$374+$N$392</f>
+        <v>5.5499999999999994E-2</v>
+      </c>
+      <c r="G403" s="9">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="H403" s="9">
+        <v>7.0699999999999999E-2</v>
+      </c>
+      <c r="I403" s="9">
+        <v>3.9800000000000002E-2</v>
+      </c>
+      <c r="J403" s="9">
+        <v>3.3799999999999997E-2</v>
+      </c>
+      <c r="L403" s="9"/>
+      <c r="N403" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>